<commit_message>
10/20 2025 VFT data integration finished
</commit_message>
<xml_diff>
--- a/raw-data/VFT Compiled data 2025/B2-25-all.xlsx
+++ b/raw-data/VFT Compiled data 2025/B2-25-all.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\VFT\VFT_github\zyao78VFTcode\raw-data\VFT Compiled data 2025\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82C0B779-AB13-463B-A5F3-1800A89DF0AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE93AA6F-ECE5-4BA2-883B-7A245990A19A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="23236" windowHeight="13875" xr2:uid="{782BA435-7A68-465F-9B70-A558FD24AC1F}"/>
   </bookViews>
@@ -1829,6 +1829,9 @@
       <c r="A24" s="9" t="s">
         <v>219</v>
       </c>
+      <c r="B24" s="6">
+        <v>1</v>
+      </c>
       <c r="E24" s="1" t="s">
         <v>189</v>
       </c>
@@ -8345,18 +8348,18 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -8536,18 +8539,18 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F20FD94B-7FF9-4F2C-BF54-A88038A3ADF3}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{62C01A46-4814-4C17-95CB-8A2CEAF90156}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{62C01A46-4814-4C17-95CB-8A2CEAF90156}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F20FD94B-7FF9-4F2C-BF54-A88038A3ADF3}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>